<commit_message>
Update spreadsheet: all 71 videos now downloaded + 11 missing ones added
</commit_message>
<xml_diff>
--- a/Chuckle_Standup_Videos.xlsx
+++ b/Chuckle_Standup_Videos.xlsx
@@ -474,7 +474,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G87"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3029,7 +3029,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F91"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3384,28 +3384,28 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>xwhJfqIyoBY</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>WHY A.I. LIES? | Gautham Govindan | Stand-Up Comedy</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="4" t="n">
         <v>226</v>
       </c>
     </row>
@@ -3436,28 +3436,28 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>vkUUB0mKv2s</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>This Comedian is All Over the Place! | Isaac Witty Stand-Up Comedy FULL SPECIAL</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="4" t="n">
         <v>201</v>
       </c>
     </row>
@@ -3644,54 +3644,54 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>zov1pWzHv0E</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>My Mom Was a Bricklayer, My Dad Was a Yoga Instructor | Dan Donohue Full Stand-U</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="4" t="n">
         <v>119</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>xNuQzXU2D_A</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>“I Smoke Weed, and I Watch Nature Shows” - Greer Barnes - Full Special</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n">
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" s="4" t="n">
         <v>112</v>
       </c>
     </row>
@@ -3774,54 +3774,54 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>txN_qF7Sk6k</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Unfiltered Matt Rife Comedy | Matt Rife Viral Crowd Work Moments</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="F29" s="4" t="n">
         <v>94</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Zy2PNTE2td4</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Hannibal Buress: Live from Chicago - Full Special</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="4" t="n">
         <v>94</v>
       </c>
     </row>
@@ -3878,54 +3878,54 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>zKUpf1Vx0vs</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Shane Gillis Live In Austin | Stand Up Comedy</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="4" t="n">
         <v>74</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>43O5Y6KXu0E</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Best Stand Up Sets Of Summer 2025 Compilation | Standup Comedy | Full Comedy Spe</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n">
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
         <v>138</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="4" t="n">
         <v>73</v>
       </c>
     </row>
@@ -4138,28 +4138,28 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>ts5FalYIzMw</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Anthony Jeselnik: Caligula - Full Special</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n">
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="F43" s="4" t="n">
         <v>55</v>
       </c>
     </row>
@@ -4190,28 +4190,28 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>zsDK94sZpXM</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>The Ones That Make You Laugh: Part 2 | Friends</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n">
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="F45" s="4" t="n">
         <v>53</v>
       </c>
     </row>
@@ -4294,28 +4294,28 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>tPi4ujR53J8</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Comedy To Brighten Your Day | Stand-Up Comedy Compilation</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n">
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="F49" s="4" t="n">
         <v>50</v>
       </c>
     </row>
@@ -4346,28 +4346,28 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>7StN8AtDsSw</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>THINKING OUT LOUD | Full show | Standup Comedy by Manoj Prabakar | English</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="n">
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="F51" s="4" t="n">
         <v>48</v>
       </c>
     </row>
@@ -4502,28 +4502,28 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>lBV8SS9zhWc</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Pete Davidson: SMD</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="n">
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="F57" s="4" t="n">
         <v>36</v>
       </c>
     </row>
@@ -4554,759 +4554,760 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>bYzT9i1zyj4</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>The Drunk Tale of Charulata - Stand Up Comedy by Kenny Sebastian</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="n">
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="F59" s="4" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>hxWLJ5ZjNNM</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Try Not To Laugh | Gabriel Iglesias</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="n">
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="F60" s="4" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>MLhCTuHqloY</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>The BEST OF STAND UP COMEDIAN Daliso Chaponda On Britain's Got Talent</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="n">
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="F61" s="4" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>TSi5zOfEaQE</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Chris D'Elia: Grow Or Die (STANDUP COMEDY SPECIAL)</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="n">
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="F62" s="2" t="n">
+      <c r="F62" s="4" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>mHKw-m0tLFw</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>60 Minutes of Jokes | Stand-up Comedy Compilation</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="n">
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="n">
         <v>77</v>
       </c>
-      <c r="F63" s="2" t="n">
+      <c r="F63" s="4" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>kZZez42HWvU</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>“I Sold Mansions to Janitors” - Tim Dillon - Full Special</t>
         </is>
       </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="n">
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="F64" s="2" t="n">
+      <c r="F64" s="4" t="n">
         <v>34</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>hFPn3WRE18w</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>This Comedy Special Will Give You Trust Issues. Chris Voth - Full Special</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="n">
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="F65" s="2" t="n">
+      <c r="F65" s="4" t="n">
         <v>34</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>tFCJLshbNdE</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>Rapid Fire Jokes You'll Never See Coming. Bobby Tessel - Full Special</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n">
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="F66" s="2" t="n">
+      <c r="F66" s="4" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>Lj_1_D712uU</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>America's Got All The Talent It Needs Right Here. @TaylorWilliamson  - Full Spec</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="n">
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="F67" s="2" t="n">
+      <c r="F67" s="4" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>k6WNXMLTB5o</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>60 Jokes That Are Pure Comedy Gold in 60 Minutes | Full Standup Comedy Compilati</t>
         </is>
       </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="n">
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="F68" s="2" t="n">
+      <c r="F68" s="4" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>p-RcbBferCw</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>Top 10 Shocking Moments | Max Amini | Stand Up Comedy</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="n">
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="F69" s="2" t="n">
+      <c r="F69" s="4" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>8qfndbEYroE</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>A Man Of Average Intelligence. Zoltan Kaszas - Full Special</t>
         </is>
       </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="n">
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="F70" s="2" t="n">
+      <c r="F70" s="4" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n">
+      <c r="A71" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>caZs9faGMH0</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>Hilarious London Moments | Max Amini | Stand Up Comedy</t>
         </is>
       </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="n">
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="F71" s="2" t="n">
+      <c r="F71" s="4" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n">
+      <c r="A72" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B72" s="5" t="inlineStr">
         <is>
           <t>BjRW9WhfGgo</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>Dan Soder: Not Special - Full Special</t>
         </is>
       </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="n">
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="F72" s="2" t="n">
+      <c r="F72" s="4" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n">
+      <c r="A73" s="4" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>9W7dIqH7wm4</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>Nikki Glaser: Perfect - Die Ganze Show | Comedy Legends | Comedy Central Deutsch</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="n">
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="F73" s="2" t="n">
+      <c r="F73" s="4" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n">
+      <c r="A74" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>EOtzzIN7ZaQ</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>21 Viral Jokes Vol. 1 | Stand Up Comedy Compilation</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="n">
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="F74" s="2" t="n">
+      <c r="F74" s="4" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n">
+      <c r="A75" s="4" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>L-i6_goqR0Y</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>Hilarious Moments in Sweden | Max Amini | Stand Up Comedy</t>
         </is>
       </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="n">
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="F75" s="2" t="n">
+      <c r="F75" s="4" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n">
+      <c r="A76" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>HHfcVW_LaT8</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>Day Spas Will Make You Uptight. David Crowe - Full Special</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="n">
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="F76" s="2" t="n">
+      <c r="F76" s="4" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n">
+      <c r="A77" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" s="5" t="inlineStr">
         <is>
           <t>JmWk1xpkeRs</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>30 Isn't Old, But It Is Almost Old. Dustin Nickerson - Full Special</t>
         </is>
       </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="n">
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F77" s="2" t="n">
+      <c r="F77" s="4" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n">
+      <c r="A78" s="4" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" s="5" t="inlineStr">
         <is>
           <t>Lhpu3GdlV3w</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr">
         <is>
           <t>The Ones That Make You Laugh | Friends</t>
         </is>
       </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="n">
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="F78" s="2" t="n">
+      <c r="F78" s="4" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n">
+      <c r="A79" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>piJdpTTo7sI</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Indian Parents Forcing Arrange marriage | Stand up comedy by Anand Rathnam </t>
         </is>
       </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="n">
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="F79" s="2" t="n">
+      <c r="F79" s="4" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n">
+      <c r="A80" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>maAepWFvb0g</t>
         </is>
       </c>
-      <c r="C80" s="3" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>Your Best Friend Sucks. Cam Bertrand - Full Special</t>
         </is>
       </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="n">
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F80" s="2" t="n">
+      <c r="F80" s="4" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n">
+      <c r="A81" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr">
         <is>
           <t>P9ZX-4U7zvs</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr">
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>Unseen Crowd Work From Comedy Special | Max Amini | Standup Comedy</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="n">
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="F81" s="2" t="n">
+      <c r="F81" s="4" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n">
+      <c r="A82" s="4" t="n">
         <v>81</v>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B82" s="5" t="inlineStr">
         <is>
           <t>zKK0-BpS-rQ</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr">
         <is>
           <t>"Come On, Who Cares?" – Chelsea Peretti - Full Special</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="n">
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F82" s="4" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n">
+      <c r="A83" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B83" s="5" t="inlineStr">
         <is>
           <t>QBzBaOl8k8A</t>
         </is>
       </c>
-      <c r="C83" s="3" t="inlineStr">
+      <c r="C83" s="5" t="inlineStr">
         <is>
           <t>Texas Vs. California | Ralph Barbosa | Stand Up Comedy</t>
         </is>
       </c>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="n">
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="F83" s="2" t="n">
+      <c r="F83" s="4" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n">
+      <c r="A84" s="4" t="n">
         <v>83</v>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>BUI0sGnx9Us</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>“The Grinch That Stole Everything”- Theo Von - Full Special</t>
         </is>
       </c>
-      <c r="D84" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="n">
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="F84" s="2" t="n">
+      <c r="F84" s="4" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n">
+      <c r="A85" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>PPnDYieoris</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>What Men Are Really Thinking About. Steve Geyer - Full Special</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="n">
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="F85" s="2" t="n">
+      <c r="F85" s="4" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" s="5" t="inlineStr">
         <is>
           <t>JpBt0W1zrDU</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>Negative Comments. Kellen Erskine - Full Special</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="n">
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="F86" s="2" t="n">
+      <c r="F86" s="4" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B87" s="5" t="inlineStr">
         <is>
           <t>Fj9-8szH6ro</t>
         </is>
       </c>
-      <c r="C87" s="3" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>Dave Chappelle's Son Meets Kevin Hart | Netflix Is A Joke</t>
         </is>
       </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>❌ No</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n">
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>✅ Yes</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F87" s="2" t="n">
+      <c r="F87" s="4" t="n">
         <v>10</v>
       </c>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
         <is>
@@ -5331,7 +5332,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>